<commit_message>
Corregeixo error en la llista de valoracions quan només seleccionava Criptos. És una mica xapussa, hauria d'arreglar-ho millor.
</commit_message>
<xml_diff>
--- a/Docs/Moviments-Arcelor.xlsx
+++ b/Docs/Moviments-Arcelor.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Repositoris\C#\_Actiu\InversionsV2\Docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FF1D927-3846-4923-A602-60020A4C88B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E3EF614-3CE0-4E87-8325-DC23B9D72197}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="0" windowWidth="23256" windowHeight="12576" xr2:uid="{3BE38316-2729-4F6D-9D30-9A2EA6E3D00C}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="12">
   <si>
     <t>Compra</t>
   </si>
@@ -55,6 +55,12 @@
   </si>
   <si>
     <t>Parts per càlcul divid</t>
+  </si>
+  <si>
+    <t>PiG</t>
+  </si>
+  <si>
+    <t>PiG amb dividends</t>
   </si>
 </sst>
 </file>
@@ -114,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -153,6 +159,11 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -477,6 +488,8 @@
     <col min="8" max="8" width="9.90625" style="16" customWidth="1"/>
     <col min="9" max="9" width="11.36328125" customWidth="1"/>
     <col min="10" max="10" width="11.26953125" customWidth="1"/>
+    <col min="12" max="12" width="11.1796875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="29" x14ac:dyDescent="0.35">
@@ -748,6 +761,7 @@
         <f t="shared" si="0"/>
         <v>527</v>
       </c>
+      <c r="J11" s="13"/>
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
@@ -772,6 +786,12 @@
       <c r="H12" s="16">
         <f>H11-D12</f>
         <v>0</v>
+      </c>
+      <c r="L12" s="18" t="s">
+        <v>10</v>
+      </c>
+      <c r="M12" s="18" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.35">
@@ -806,6 +826,14 @@
         <f>E$16/H$16*I13</f>
         <v>169.60813559322034</v>
       </c>
+      <c r="L13" s="7">
+        <f>(K17*E17)+(K14*E14)-(D13*E13)-F13-F14-(F17/D17*K17)</f>
+        <v>-12360.491456869011</v>
+      </c>
+      <c r="M13" s="13">
+        <f>L13+J13</f>
+        <v>-12190.883321275791</v>
+      </c>
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
@@ -832,6 +860,10 @@
         <v>952</v>
       </c>
       <c r="J14" s="13"/>
+      <c r="K14">
+        <f>D14</f>
+        <v>648</v>
+      </c>
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15" s="1">
@@ -865,18 +897,8 @@
         <f>E$16/H$16*I15</f>
         <v>124.71186440677965</v>
       </c>
-      <c r="K15">
-        <f>H17</f>
-        <v>400</v>
-      </c>
-      <c r="L15" s="13">
-        <f>J15/D15*K15</f>
-        <v>71.263922518159802</v>
-      </c>
-      <c r="M15" s="7">
-        <f>F15/D15*K15</f>
-        <v>5.7485714285714282</v>
-      </c>
+      <c r="L15" s="13"/>
+      <c r="M15" s="7"/>
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16" s="1">
@@ -929,6 +951,10 @@
         <v>400</v>
       </c>
       <c r="J17" s="13"/>
+      <c r="K17">
+        <f>D13-K14</f>
+        <v>952</v>
+      </c>
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18" s="1">
@@ -982,13 +1008,13 @@
         <f t="shared" ref="H19:H24" si="1">H18+D19</f>
         <v>1560</v>
       </c>
-      <c r="I19" s="10">
-        <f>H21</f>
-        <v>400</v>
+      <c r="I19" s="19">
+        <f>H21-I20</f>
+        <v>308</v>
       </c>
       <c r="J19" s="14">
         <f>E$25/H$25*I19</f>
-        <v>98.351578947368424</v>
+        <v>75.730715789473692</v>
       </c>
       <c r="L19" s="13"/>
       <c r="M19" s="7"/>
@@ -997,7 +1023,7 @@
       <c r="A20" s="1">
         <v>190</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C20" s="2">
@@ -1017,7 +1043,14 @@
         <f t="shared" si="1"/>
         <v>1652</v>
       </c>
-      <c r="J20" s="13"/>
+      <c r="I20" s="10">
+        <f>D20</f>
+        <v>92</v>
+      </c>
+      <c r="J20" s="14">
+        <f>E$25/H$25*I20</f>
+        <v>22.620863157894739</v>
+      </c>
       <c r="L20" s="13"/>
       <c r="M20" s="7"/>
     </row>
@@ -1172,7 +1205,8 @@
         <f>H24+D25</f>
         <v>1900</v>
       </c>
-      <c r="J25" s="7"/>
+      <c r="I25" s="16"/>
+      <c r="J25" s="20"/>
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26" s="1">

</xml_diff>